<commit_message>
Aşama 4: Optimizasyon (Pyomo + HiGHS)
- Ön adımlar: borç deflasyonu bağımsız testlerle doğrulandı (hata yok); başabaş fiyat
  metriği; düzenleyici araştırma (depolamalı tesis, şebekeden şarj, yardımcı kaynak) ve
  config anahtarları
- Finansal model: ekonomik kesinti, batarya kancası düzeltmesi (deşarj geliri), 20. yıl
  yenileme ve 6 USD/MWh yıpranma
- B1 batarya arbitrajı LP; B2 hibrit + batarya LP ve saatlik şebeke gölge fiyatı
- B3 kapasite MILP (türbin tamsayı, yatırım ikili, seviyelendirilmiş fiyat, vergi düzeltmeli
  yıllıklandırma); temsilî günler (k-means + medoid + moment eşleştirme) vs tam yıl
- B4 ayrıntılı değerlendirme (dispatch kancası), 6 senaryo + pişmanlık, şebeke boyutu ve
  katkı payı tavanı, GES × batarya ızgarası, başabaş fiyat
- docs/04_optimizasyon.md, README, CLAUDE.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/03_finans/nakit_akisi_b.xlsx
+++ b/outputs/03_finans/nakit_akisi_b.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-7.97</v>
+        <v>-7.43</v>
       </c>
     </row>
     <row r="5">
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.76</v>
+        <v>5.85</v>
       </c>
     </row>
     <row r="6">
@@ -509,7 +509,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6.2 / 8.9</t>
+          <t>6.4 / 9.1</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>48.6 / 49.0 / 50.1</t>
+          <t>48.6 / 49.0 / 53.8</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>51</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="10">
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2.2</v>
+        <v>9.58</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>44.92</v>
+        <v>45.29</v>
       </c>
     </row>
     <row r="13">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>56.9</v>
+        <v>57.3</v>
       </c>
     </row>
   </sheetData>
@@ -596,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z35"/>
+  <dimension ref="A1:AD35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -608,23 +608,27 @@
     <col width="16.2" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="29.7" customWidth="1" min="10" max="10"/>
-    <col width="19.8" customWidth="1" min="11" max="11"/>
-    <col width="18.9" customWidth="1" min="12" max="12"/>
-    <col width="27.9" customWidth="1" min="13" max="13"/>
-    <col width="15.3" customWidth="1" min="14" max="14"/>
-    <col width="22.5" customWidth="1" min="15" max="15"/>
-    <col width="16.2" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="19.8" customWidth="1" min="18" max="18"/>
-    <col width="13.5" customWidth="1" min="19" max="19"/>
-    <col width="17.1" customWidth="1" min="20" max="20"/>
-    <col width="26.1" customWidth="1" min="21" max="21"/>
-    <col width="13.5" customWidth="1" min="22" max="22"/>
-    <col width="17.1" customWidth="1" min="23" max="23"/>
-    <col width="22.5" customWidth="1" min="24" max="24"/>
-    <col width="27.9" customWidth="1" min="25" max="25"/>
-    <col width="33.3" customWidth="1" min="26" max="26"/>
+    <col width="18.9" customWidth="1" min="10" max="10"/>
+    <col width="15.3" customWidth="1" min="11" max="11"/>
+    <col width="19.8" customWidth="1" min="12" max="12"/>
+    <col width="29.7" customWidth="1" min="13" max="13"/>
+    <col width="19.8" customWidth="1" min="14" max="14"/>
+    <col width="18.9" customWidth="1" min="15" max="15"/>
+    <col width="27.9" customWidth="1" min="16" max="16"/>
+    <col width="20.7" customWidth="1" min="17" max="17"/>
+    <col width="15.3" customWidth="1" min="18" max="18"/>
+    <col width="22.5" customWidth="1" min="19" max="19"/>
+    <col width="16.2" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="34.2" customWidth="1" min="22" max="22"/>
+    <col width="13.5" customWidth="1" min="23" max="23"/>
+    <col width="17.1" customWidth="1" min="24" max="24"/>
+    <col width="26.1" customWidth="1" min="25" max="25"/>
+    <col width="13.5" customWidth="1" min="26" max="26"/>
+    <col width="17.1" customWidth="1" min="27" max="27"/>
+    <col width="22.5" customWidth="1" min="28" max="28"/>
+    <col width="27.9" customWidth="1" min="29" max="29"/>
+    <col width="33.3" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -675,85 +679,105 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>BESS geliri [bin USD]</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>BESS deşarj [MWh]</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>BESS'ten satılan [MWh]</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Eşzamanlılık düzeltmesi [bin USD]</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Toplam gelir [bin USD]</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Dengesizlik [bin USD]</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>İşletme-bakım + arazi [bin USD]</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>BESS yıpranma [bin USD]</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Sigorta [bin USD]</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>TEİAŞ bedelleri [bin USD]</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>FAVÖK [bin USD]</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Amortisman [bin USD]</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Augmentation [bin USD]</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>BESS augmentation + yenileme [bin USD]</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Söküm [bin USD]</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Vergi [bin USD]</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Serbest nakit akışı [bin USD]</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>CAPEX [bin USD]</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>İskonto çarpanı</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>İndirgenmiş SNA [bin USD]</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Borç servisi, nominal [bin USD]</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Öz kaynak nakit akışı, reel [bin USD]</t>
         </is>
@@ -823,22 +847,34 @@
         <v>0</v>
       </c>
       <c r="U2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="3" t="n">
         <v>-31600</v>
       </c>
-      <c r="V2" s="3" t="n">
+      <c r="Z2" s="3" t="n">
         <v>-31600</v>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="AA2" s="4" t="n">
         <v>0.9345794392523364</v>
       </c>
-      <c r="X2" s="3" t="n">
+      <c r="AB2" s="3" t="n">
         <v>-29532.71028037383</v>
       </c>
-      <c r="Y2" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z2" s="3" t="n">
-        <v>-13633.50832971958</v>
+      <c r="AC2" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD2" s="3" t="n">
+        <v>-13484.94121338748</v>
       </c>
     </row>
     <row r="3">
@@ -905,22 +941,34 @@
         <v>0</v>
       </c>
       <c r="U3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="3" t="n">
         <v>-47400</v>
       </c>
-      <c r="V3" s="3" t="n">
+      <c r="Z3" s="3" t="n">
         <v>-47400</v>
       </c>
-      <c r="W3" s="4" t="n">
+      <c r="AA3" s="4" t="n">
         <v>0.8734387282732116</v>
       </c>
-      <c r="X3" s="3" t="n">
+      <c r="AB3" s="3" t="n">
         <v>-41400.99572015023</v>
       </c>
-      <c r="Y3" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z3" s="3" t="n">
-        <v>-20450.26249457937</v>
+      <c r="AC3" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD3" s="3" t="n">
+        <v>-20227.41182008122</v>
       </c>
     </row>
     <row r="4">
@@ -939,70 +987,82 @@
         <v>164978.4686679672</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>6520.410581349131</v>
+        <v>17629.01408760873</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>203491.1043931759</v>
+        <v>192382.5008869163</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1807.111015193316</v>
+        <v>1803.464073320454</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>8963.963352935398</v>
+        <v>8976.141491058062</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>-446.6808160106663</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>10771.07436812871</v>
+        <v>0</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>-394.7007544212823</v>
+        <v>0</v>
       </c>
       <c r="M4" s="3" t="n">
+        <v>-429.3244567076158</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>10779.60556437852</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>-395.1149411087316</v>
+      </c>
+      <c r="P4" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N4" s="3" t="n">
+      <c r="Q4" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R4" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O4" s="3" t="n">
-        <v>-946.7661966940684</v>
-      </c>
-      <c r="P4" s="3" t="n">
-        <v>6978.107417013362</v>
-      </c>
-      <c r="Q4" s="3" t="n">
+      <c r="S4" s="3" t="n">
+        <v>-904.5535033702819</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>7028.437119899504</v>
+      </c>
+      <c r="U4" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R4" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S4" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T4" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U4" s="3" t="n">
-        <v>6978.107417013362</v>
-      </c>
       <c r="V4" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W4" s="4" t="n">
+      <c r="W4" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>7028.437119899504</v>
+      </c>
+      <c r="Z4" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA4" s="4" t="n">
         <v>0.8162978768908519</v>
       </c>
-      <c r="X4" s="3" t="n">
-        <v>5696.214269224314</v>
-      </c>
-      <c r="Y4" s="3" t="n">
-        <v>-5313.649277033207</v>
-      </c>
-      <c r="Z4" s="3" t="n">
-        <v>2043.855828526176</v>
+      <c r="AB4" s="3" t="n">
+        <v>5737.298298834819</v>
+      </c>
+      <c r="AC4" s="3" t="n">
+        <v>-5352.894475810855</v>
+      </c>
+      <c r="AD4" s="3" t="n">
+        <v>2057.742462945966</v>
       </c>
     </row>
     <row r="5">
@@ -1021,70 +1081,82 @@
         <v>164483.5332619633</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>6352.447286551739</v>
+        <v>18761.44626668967</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>202938.9670504366</v>
+        <v>190529.9680702987</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1740.532698733995</v>
+        <v>1734.824159938062</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>8918.489001255588</v>
+        <v>8930.191809833765</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>-445.6280317224587</v>
+        <v>0</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>10659.02169998958</v>
+        <v>0</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>-391.5502140249035</v>
+        <v>0</v>
       </c>
       <c r="M5" s="3" t="n">
+        <v>-426.2828574982024</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>10665.01596977183</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>-391.9041555921119</v>
+      </c>
+      <c r="P5" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N5" s="3" t="n">
+      <c r="Q5" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R5" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O5" s="3" t="n">
-        <v>-944.6680747916589</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>6871.303411173021</v>
-      </c>
-      <c r="Q5" s="3" t="n">
+      <c r="S5" s="3" t="n">
+        <v>-897.5138786671349</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>6924.09793551258</v>
+      </c>
+      <c r="U5" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R5" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S5" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T5" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U5" s="3" t="n">
-        <v>6871.303411173021</v>
-      </c>
       <c r="V5" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W5" s="4" t="n">
+      <c r="W5" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>6924.09793551258</v>
+      </c>
+      <c r="Z5" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA5" s="4" t="n">
         <v>0.7628952120475251</v>
       </c>
-      <c r="X5" s="3" t="n">
-        <v>5242.084472909724</v>
-      </c>
-      <c r="Y5" s="3" t="n">
-        <v>-5361.126741559908</v>
-      </c>
-      <c r="Z5" s="3" t="n">
-        <v>2014.387182803612</v>
+      <c r="AB5" s="3" t="n">
+        <v>5282.361162750701</v>
+      </c>
+      <c r="AC5" s="3" t="n">
+        <v>-5403.32309421738</v>
+      </c>
+      <c r="AD5" s="3" t="n">
+        <v>2028.953894244936</v>
       </c>
     </row>
     <row r="6">
@@ -1103,70 +1175,82 @@
         <v>163990.0826621774</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>6186.884474126875</v>
+        <v>19553.86234247124</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>202387.0398577005</v>
+        <v>189020.0619893561</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1674.41571835339</v>
+        <v>1667.438731498082</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>8872.809648098351</v>
+        <v>8884.352047379742</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>-444.5747585168736</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>10547.22536645174</v>
+        <v>0</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>-388.4007002910018</v>
+        <v>0</v>
       </c>
       <c r="M6" s="3" t="n">
+        <v>-423.7021316317376</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>10551.79077887782</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>-388.7228565251513</v>
+      </c>
+      <c r="P6" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N6" s="3" t="n">
+      <c r="Q6" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R6" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O6" s="3" t="n">
-        <v>-942.5707514592617</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>6764.753914701477</v>
-      </c>
-      <c r="Q6" s="3" t="n">
+      <c r="S6" s="3" t="n">
+        <v>-891.776235559553</v>
+      </c>
+      <c r="T6" s="3" t="n">
+        <v>6819.791686793119</v>
+      </c>
+      <c r="U6" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R6" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S6" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T6" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U6" s="3" t="n">
-        <v>6764.753914701477</v>
-      </c>
       <c r="V6" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W6" s="4" t="n">
+      <c r="W6" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y6" s="3" t="n">
+        <v>6819.791686793119</v>
+      </c>
+      <c r="Z6" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA6" s="4" t="n">
         <v>0.7129861794836683</v>
       </c>
-      <c r="X6" s="3" t="n">
-        <v>4823.176048790195</v>
-      </c>
-      <c r="Y6" s="3" t="n">
-        <v>-5407.865552169205</v>
-      </c>
-      <c r="Z6" s="3" t="n">
-        <v>1984.988759600914</v>
+      <c r="AB6" s="3" t="n">
+        <v>4862.417219641107</v>
+      </c>
+      <c r="AC6" s="3" t="n">
+        <v>-5452.954566635299</v>
+      </c>
+      <c r="AD6" s="3" t="n">
+        <v>2000.174412932613</v>
       </c>
     </row>
     <row r="7">
@@ -1185,70 +1269,82 @@
         <v>163498.1124141908</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>6023.722696039537</v>
+        <v>20300.09252886552</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>201835.312179453</v>
+        <v>187558.942346627</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>1608.758995856046</v>
+        <v>1600.737834203053</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>8826.931891111859</v>
+        <v>8838.43587697166</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>-443.520973993735</v>
+        <v>0</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>10435.6908869679</v>
+        <v>0</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>-385.2524555615952</v>
+        <v>0</v>
       </c>
       <c r="M7" s="3" t="n">
+        <v>-421.1519309003343</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>10439.17371117471</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>-385.5521917629275</v>
+      </c>
+      <c r="P7" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N7" s="3" t="n">
+      <c r="Q7" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R7" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O7" s="3" t="n">
-        <v>-940.4741862819212</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>6658.464245124388</v>
-      </c>
-      <c r="Q7" s="3" t="n">
+      <c r="S7" s="3" t="n">
+        <v>-886.2239809171826</v>
+      </c>
+      <c r="T7" s="3" t="n">
+        <v>6715.897538494602</v>
+      </c>
+      <c r="U7" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R7" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S7" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T7" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U7" s="3" t="n">
-        <v>6658.464245124388</v>
-      </c>
       <c r="V7" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W7" s="4" t="n">
+      <c r="W7" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y7" s="3" t="n">
+        <v>6715.897538494602</v>
+      </c>
+      <c r="Z7" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA7" s="4" t="n">
         <v>0.6663422238165123</v>
       </c>
-      <c r="X7" s="3" t="n">
-        <v>4436.815872298919</v>
-      </c>
-      <c r="Y7" s="3" t="n">
-        <v>-5453.808780566352</v>
-      </c>
-      <c r="Z7" s="3" t="n">
-        <v>1955.662026094141</v>
+      <c r="AB7" s="3" t="n">
+        <v>4475.086100724335</v>
+      </c>
+      <c r="AC7" s="3" t="n">
+        <v>-5502.036584120528</v>
+      </c>
+      <c r="AD7" s="3" t="n">
+        <v>1971.50863560743</v>
       </c>
     </row>
     <row r="8">
@@ -1267,70 +1363,82 @@
         <v>163007.6180769483</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>5862.837016937264</v>
+        <v>20677.5462694081</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>201283.8989090062</v>
+        <v>186469.1896565353</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>1543.561851345257</v>
+        <v>1535.108665794123</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>8780.861747595869</v>
+        <v>8792.658214028505</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>-442.466950257473</v>
+        <v>0</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>10324.42359894113</v>
+        <v>0</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>-382.1057069307399</v>
+        <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
+        <v>-419.2410517061745</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>10327.76687982263</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>-382.4085018770226</v>
+      </c>
+      <c r="P8" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N8" s="3" t="n">
+      <c r="Q8" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R8" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O8" s="3" t="n">
-        <v>-938.3788158542234</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>6552.439076156164</v>
-      </c>
-      <c r="Q8" s="3" t="n">
+      <c r="S8" s="3" t="n">
+        <v>-882.0829206948342</v>
+      </c>
+      <c r="T8" s="3" t="n">
+        <v>6611.77545725077</v>
+      </c>
+      <c r="U8" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R8" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S8" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T8" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U8" s="3" t="n">
-        <v>6552.439076156164</v>
-      </c>
       <c r="V8" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W8" s="4" t="n">
+      <c r="W8" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X8" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y8" s="3" t="n">
+        <v>6611.77545725077</v>
+      </c>
+      <c r="Z8" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA8" s="4" t="n">
         <v>0.6227497418845909</v>
       </c>
-      <c r="X8" s="3" t="n">
-        <v>4080.529743390758</v>
-      </c>
-      <c r="Y8" s="3" t="n">
-        <v>-5498.896913140829</v>
-      </c>
-      <c r="Z8" s="3" t="n">
-        <v>1926.408271823255</v>
+      <c r="AB8" s="3" t="n">
+        <v>4117.48145940179</v>
+      </c>
+      <c r="AC8" s="3" t="n">
+        <v>-5549.968421358462</v>
+      </c>
+      <c r="AD8" s="3" t="n">
+        <v>1942.77996855109</v>
       </c>
     </row>
     <row r="9">
@@ -1349,70 +1457,82 @@
         <v>162518.5952227174</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>5704.336953600617</v>
+        <v>21274.79079940083</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>200732.680528867</v>
+        <v>185162.2266830668</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>1478.821744784261</v>
+        <v>1469.700014575054</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>8734.603073099674</v>
+        <v>8746.638426521182</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>-441.4124863595916</v>
+        <v>0</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>10213.42481788393</v>
+        <v>0</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>-378.9605578196721</v>
+        <v>0</v>
       </c>
       <c r="M9" s="3" t="n">
+        <v>-416.9458857178615</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>10216.33844109624</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>-379.2595373523483</v>
+      </c>
+      <c r="P9" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N9" s="3" t="n">
+      <c r="Q9" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R9" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O9" s="3" t="n">
-        <v>-936.2841860096946</v>
-      </c>
-      <c r="P9" s="3" t="n">
-        <v>6446.680074054566</v>
-      </c>
-      <c r="Q9" s="3" t="n">
+      <c r="S9" s="3" t="n">
+        <v>-877.1164613956539</v>
+      </c>
+      <c r="T9" s="3" t="n">
+        <v>6508.462442348234</v>
+      </c>
+      <c r="U9" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R9" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S9" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T9" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U9" s="3" t="n">
-        <v>6446.680074054566</v>
-      </c>
       <c r="V9" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W9" s="4" t="n">
+      <c r="W9" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y9" s="3" t="n">
+        <v>6508.462442348234</v>
+      </c>
+      <c r="Z9" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA9" s="4" t="n">
         <v>0.5820091045650382</v>
       </c>
-      <c r="X9" s="3" t="n">
-        <v>3752.026497317772</v>
-      </c>
-      <c r="Y9" s="3" t="n">
-        <v>-5543.065642073422</v>
-      </c>
-      <c r="Z9" s="3" t="n">
-        <v>1897.227956530934</v>
+      <c r="AB9" s="3" t="n">
+        <v>3787.984398166277</v>
+      </c>
+      <c r="AC9" s="3" t="n">
+        <v>-5597.57185965195</v>
+      </c>
+      <c r="AD9" s="3" t="n">
+        <v>1914.274533659032</v>
       </c>
     </row>
     <row r="10">
@@ -1431,70 +1551,82 @@
         <v>162031.0394370493</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>5548.286854664122</v>
+        <v>21077.25579105586</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>200181.5827308366</v>
+        <v>184652.6137944449</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>1472.623527099198</v>
+        <v>1463.538509791885</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>8711.361479163919</v>
+        <v>8723.376888222248</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>-440.3573775706585</v>
+        <v>0</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>10183.98500626312</v>
+        <v>0</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>-377.9069297085408</v>
+        <v>0</v>
       </c>
       <c r="M10" s="3" t="n">
+        <v>-415.9279819837428</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>10186.91539801413</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>-378.2058457247277</v>
+      </c>
+      <c r="P10" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N10" s="3" t="n">
+      <c r="Q10" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R10" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O10" s="3" t="n">
-        <v>-934.1900143771791</v>
-      </c>
-      <c r="P10" s="3" t="n">
-        <v>6420.388062177397</v>
-      </c>
-      <c r="Q10" s="3" t="n">
+      <c r="S10" s="3" t="n">
+        <v>-875.1799324188905</v>
+      </c>
+      <c r="T10" s="3" t="n">
+        <v>6482.029619870515</v>
+      </c>
+      <c r="U10" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R10" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S10" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T10" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U10" s="3" t="n">
-        <v>6420.388062177397</v>
-      </c>
       <c r="V10" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W10" s="4" t="n">
+      <c r="W10" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y10" s="3" t="n">
+        <v>6482.029619870515</v>
+      </c>
+      <c r="Z10" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA10" s="4" t="n">
         <v>0.5439337425841478</v>
       </c>
-      <c r="X10" s="3" t="n">
-        <v>3492.265707502736</v>
-      </c>
-      <c r="Y10" s="3" t="n">
-        <v>-5657.866809417757</v>
-      </c>
-      <c r="Z10" s="3" t="n">
-        <v>1889.97364076585</v>
+      <c r="AB10" s="3" t="n">
+        <v>3525.794630677471</v>
+      </c>
+      <c r="AC10" s="3" t="n">
+        <v>-5713.608349512475</v>
+      </c>
+      <c r="AD10" s="3" t="n">
+        <v>1906.981366376452</v>
       </c>
     </row>
     <row r="11">
@@ -1513,70 +1645,82 @@
         <v>161544.9463187381</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5394.468051065776</v>
+        <v>20881.95522391883</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>199630.8142653815</v>
+        <v>184143.3270925285</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>1466.439582310823</v>
+        <v>1457.391172140343</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>8688.140086874428</v>
+        <v>8700.135441201122</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>-439.3020624645724</v>
+        <v>0</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>10154.57966918525</v>
+        <v>0</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>-376.8543951211935</v>
+        <v>0</v>
       </c>
       <c r="M11" s="3" t="n">
+        <v>-414.9101092856523</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>10157.52661334147</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>-377.1532410908517</v>
+      </c>
+      <c r="P11" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N11" s="3" t="n">
+      <c r="Q11" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R11" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O11" s="3" t="n">
-        <v>-932.0970942084497</v>
-      </c>
-      <c r="P11" s="3" t="n">
-        <v>6394.128179855607</v>
-      </c>
-      <c r="Q11" s="3" t="n">
+      <c r="S11" s="3" t="n">
+        <v>-873.2446429516083</v>
+      </c>
+      <c r="T11" s="3" t="n">
+        <v>6455.628729299007</v>
+      </c>
+      <c r="U11" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R11" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S11" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T11" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U11" s="3" t="n">
-        <v>6394.128179855607</v>
-      </c>
       <c r="V11" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W11" s="4" t="n">
+      <c r="W11" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y11" s="3" t="n">
+        <v>6455.628729299007</v>
+      </c>
+      <c r="Z11" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA11" s="4" t="n">
         <v>0.5083492921347176</v>
       </c>
-      <c r="X11" s="3" t="n">
-        <v>3250.450534048248</v>
-      </c>
-      <c r="Y11" s="3" t="n">
-        <v>-5774.973399737062</v>
-      </c>
-      <c r="Z11" s="3" t="n">
-        <v>1882.728189972425</v>
+      <c r="AB11" s="3" t="n">
+        <v>3281.714294823696</v>
+      </c>
+      <c r="AC11" s="3" t="n">
+        <v>-5831.977778888319</v>
+      </c>
+      <c r="AD11" s="3" t="n">
+        <v>1899.697009531494</v>
       </c>
     </row>
     <row r="12">
@@ -1595,70 +1739,82 @@
         <v>161060.3114797819</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>5242.990466991405</v>
+        <v>20688.9513362722</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>199080.2553305112</v>
+        <v>183634.2944612303</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>1460.269204556251</v>
+        <v>1451.257318135391</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>8664.938934279244</v>
+        <v>8676.914069010307</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>-438.2463095527371</v>
+        <v>0</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>10125.20813883549</v>
+        <v>0</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>-375.8029414622948</v>
+        <v>0</v>
       </c>
       <c r="M12" s="3" t="n">
+        <v>-413.8921156298848</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>10128.1713871457</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>-376.1017091231201</v>
+      </c>
+      <c r="P12" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N12" s="3" t="n">
+      <c r="Q12" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R12" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O12" s="3" t="n">
-        <v>-930.0049702559425</v>
-      </c>
-      <c r="P12" s="3" t="n">
-        <v>6367.900227117258</v>
-      </c>
-      <c r="Q12" s="3" t="n">
+      <c r="S12" s="3" t="n">
+        <v>-871.3103189526752</v>
+      </c>
+      <c r="T12" s="3" t="n">
+        <v>6429.259359069902</v>
+      </c>
+      <c r="U12" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R12" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S12" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T12" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U12" s="3" t="n">
-        <v>6367.900227117258</v>
-      </c>
       <c r="V12" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W12" s="4" t="n">
+      <c r="W12" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X12" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y12" s="3" t="n">
+        <v>6429.259359069902</v>
+      </c>
+      <c r="Z12" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA12" s="4" t="n">
         <v>0.4750927963875865</v>
       </c>
-      <c r="X12" s="3" t="n">
-        <v>3025.343526018285</v>
-      </c>
-      <c r="Y12" s="3" t="n">
-        <v>-5894.429487980112</v>
-      </c>
-      <c r="Z12" s="3" t="n">
-        <v>1875.491548975735</v>
+      <c r="AB12" s="3" t="n">
+        <v>3054.494807601582</v>
+      </c>
+      <c r="AC12" s="3" t="n">
+        <v>-5952.724620872793</v>
+      </c>
+      <c r="AD12" s="3" t="n">
+        <v>1892.421349568231</v>
       </c>
     </row>
     <row r="13">
@@ -1677,70 +1833,82 @@
         <v>160577.1305453426</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>5094.026136811474</v>
+        <v>20498.35664189593</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>198529.7240546631</v>
+        <v>183125.3935495787</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1454.111916969786</v>
+        <v>1445.136493636362</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>8641.75777470118</v>
+        <v>8653.712449093095</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>-437.1897654552124</v>
+        <v>0</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>10095.86969167097</v>
+        <v>0</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>-374.7525493274429</v>
+        <v>0</v>
       </c>
       <c r="M13" s="3" t="n">
+        <v>-412.8737589317065</v>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>10098.84894272946</v>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>-375.051227836451</v>
+      </c>
+      <c r="P13" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N13" s="3" t="n">
+      <c r="Q13" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R13" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O13" s="3" t="n">
-        <v>-927.9129514077199</v>
-      </c>
-      <c r="P13" s="3" t="n">
-        <v>6341.704190935803</v>
-      </c>
-      <c r="Q13" s="3" t="n">
+      <c r="S13" s="3" t="n">
+        <v>-869.376495488399</v>
+      </c>
+      <c r="T13" s="3" t="n">
+        <v>6402.921219404607</v>
+      </c>
+      <c r="U13" s="3" t="n">
         <v>-7900</v>
       </c>
-      <c r="R13" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="S13" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="T13" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="U13" s="3" t="n">
-        <v>6341.704190935803</v>
-      </c>
       <c r="V13" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W13" s="4" t="n">
+      <c r="W13" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X13" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y13" s="3" t="n">
+        <v>6402.921219404607</v>
+      </c>
+      <c r="Z13" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA13" s="4" t="n">
         <v>0.444011959240735</v>
       </c>
-      <c r="X13" s="3" t="n">
-        <v>2815.792502742586</v>
-      </c>
-      <c r="Y13" s="3" t="n">
-        <v>-6016.280103117766</v>
-      </c>
-      <c r="Z13" s="3" t="n">
-        <v>1868.263714181593</v>
+      <c r="AB13" s="3" t="n">
+        <v>2842.973595491916</v>
+      </c>
+      <c r="AC13" s="3" t="n">
+        <v>-6075.894231670859</v>
+      </c>
+      <c r="AD13" s="3" t="n">
+        <v>1885.154306532895</v>
       </c>
     </row>
     <row r="14">
@@ -1759,70 +1927,82 @@
         <v>160095.3991537065</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>4947.374815298646</v>
+        <v>20309.99350936744</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>197979.4108863093</v>
+        <v>182616.7921922405</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>1447.969152074552</v>
+        <v>1439.030126144554</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>8618.599754029989</v>
+        <v>8630.533757762574</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>-436.1328006302674</v>
+        <v>0</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>10066.56890610454</v>
+        <v>0</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>-373.7033732026906</v>
+        <v>0</v>
       </c>
       <c r="M14" s="3" t="n">
+        <v>-411.855352897365</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>10069.56388390713</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>-374.0019528333941</v>
+      </c>
+      <c r="P14" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N14" s="3" t="n">
+      <c r="Q14" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R14" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O14" s="3" t="n">
-        <v>-925.8217613679752</v>
-      </c>
-      <c r="P14" s="3" t="n">
-        <v>6315.543771533875</v>
-      </c>
-      <c r="Q14" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R14" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S14" s="3" t="n">
-        <v>-0</v>
+        <v>-867.4438103305138</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>-0</v>
+        <v>6376.618120743221</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>6315.543771533875</v>
+        <v>-0</v>
       </c>
       <c r="V14" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W14" s="4" t="n">
+      <c r="W14" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X14" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Y14" s="3" t="n">
+        <v>6376.618120743221</v>
+      </c>
+      <c r="Z14" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA14" s="4" t="n">
         <v>0.4149644478885374</v>
       </c>
-      <c r="X14" s="3" t="n">
-        <v>2620.726134270446</v>
-      </c>
-      <c r="Y14" s="3" t="n">
-        <v>-6140.57478188086</v>
-      </c>
-      <c r="Z14" s="3" t="n">
-        <v>1861.04570653063</v>
+      <c r="AB14" s="3" t="n">
+        <v>2646.069817870253</v>
+      </c>
+      <c r="AC14" s="3" t="n">
+        <v>-6201.536846702267</v>
+      </c>
+      <c r="AD14" s="3" t="n">
+        <v>1877.896931776589</v>
       </c>
     </row>
     <row r="15">
@@ -1841,70 +2021,82 @@
         <v>159615.1129562454</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>4802.885192064398</v>
+        <v>20123.74562019929</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>197429.4573793429</v>
+        <v>182108.596951208</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>1441.842234953434</v>
+        <v>1432.939503857521</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>8595.468524072834</v>
+        <v>8607.381660865882</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>-435.0757035818707</v>
+        <v>0</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>10037.31075902627</v>
+        <v>0</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>-372.655585661982</v>
+        <v>0</v>
       </c>
       <c r="M15" s="3" t="n">
+        <v>-410.837138504273</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>10040.3211647234</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>-372.9540565117857</v>
+      </c>
+      <c r="P15" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N15" s="3" t="n">
+      <c r="Q15" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R15" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O15" s="3" t="n">
-        <v>-923.731938041503</v>
-      </c>
-      <c r="P15" s="3" t="n">
-        <v>6289.423235322783</v>
-      </c>
-      <c r="Q15" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R15" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S15" s="3" t="n">
-        <v>-0</v>
+        <v>-865.5126684145904</v>
       </c>
       <c r="T15" s="3" t="n">
-        <v>-1268.941935249322</v>
+        <v>6350.354439797027</v>
       </c>
       <c r="U15" s="3" t="n">
-        <v>5020.48130007346</v>
+        <v>-0</v>
       </c>
       <c r="V15" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W15" s="4" t="n">
+      <c r="W15" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X15" s="3" t="n">
+        <v>-1376.318482633128</v>
+      </c>
+      <c r="Y15" s="3" t="n">
+        <v>4974.035957163899</v>
+      </c>
+      <c r="Z15" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA15" s="4" t="n">
         <v>0.3878172410173246</v>
       </c>
-      <c r="X15" s="3" t="n">
-        <v>1947.029206373561</v>
-      </c>
-      <c r="Y15" s="3" t="n">
-        <v>-5892.014370879227</v>
-      </c>
-      <c r="Z15" s="3" t="n">
-        <v>1092.993419116214</v>
+      <c r="AB15" s="3" t="n">
+        <v>1929.016901628271</v>
+      </c>
+      <c r="AC15" s="3" t="n">
+        <v>-5844.495418277952</v>
+      </c>
+      <c r="AD15" s="3" t="n">
+        <v>1081.205416985813</v>
       </c>
     </row>
     <row r="16">
@@ -1923,70 +2115,82 @@
         <v>159136.2676173767</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>4660.527405689914</v>
+        <v>19939.61084153873</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>196879.8836787728</v>
+        <v>181600.800242924</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>1435.731046835439</v>
+        <v>1426.864500405997</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>8572.363640013562</v>
+        <v>8584.255773256284</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>-434.0185212415701</v>
+        <v>0</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>10008.094686849</v>
+        <v>0</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>-371.6091665372513</v>
+        <v>0</v>
       </c>
       <c r="M16" s="3" t="n">
+        <v>-409.819108222291</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>10011.12027366228</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>-371.9075209383713</v>
+      </c>
+      <c r="P16" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N16" s="3" t="n">
+      <c r="Q16" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R16" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O16" s="3" t="n">
-        <v>-921.6435579793366</v>
-      </c>
-      <c r="P16" s="3" t="n">
-        <v>6263.341962332414</v>
-      </c>
-      <c r="Q16" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R16" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S16" s="3" t="n">
-        <v>-0</v>
+        <v>-863.5830409231113</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>-1565.835490583104</v>
+        <v>6324.129711800799</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>4697.506471749311</v>
+        <v>-0</v>
       </c>
       <c r="V16" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W16" s="4" t="n">
+      <c r="W16" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X16" s="3" t="n">
+        <v>-1581.0324279502</v>
+      </c>
+      <c r="Y16" s="3" t="n">
+        <v>4743.0972838506</v>
+      </c>
+      <c r="Z16" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA16" s="4" t="n">
         <v>0.3624460196423595</v>
       </c>
-      <c r="X16" s="3" t="n">
-        <v>1702.592522929762</v>
-      </c>
-      <c r="Y16" s="3" t="n">
-        <v>-4797.523264020599</v>
-      </c>
-      <c r="Z16" s="3" t="n">
-        <v>1559.077729205146</v>
+      <c r="AB16" s="3" t="n">
+        <v>1719.116731308136</v>
+      </c>
+      <c r="AC16" s="3" t="n">
+        <v>-4845.334049584205</v>
+      </c>
+      <c r="AD16" s="3" t="n">
+        <v>1573.39503152432</v>
       </c>
     </row>
     <row r="17">
@@ -2005,70 +2209,82 @@
         <v>158658.8588145245</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>4520.424849784914</v>
+        <v>19757.70330921326</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>196330.5567144902</v>
+        <v>181093.2782550619</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>1429.632684185236</v>
+        <v>1420.802253402195</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>8549.273087304171</v>
+        <v>8561.144090497433</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>-432.9609226147603</v>
+        <v>0</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>9978.905771489406</v>
+        <v>0</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>-370.5635771758716</v>
+        <v>0</v>
       </c>
       <c r="M17" s="3" t="n">
+        <v>-408.8009339426098</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>9981.94634389963</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>-370.8618086879413</v>
+      </c>
+      <c r="P17" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N17" s="3" t="n">
+      <c r="Q17" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R17" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O17" s="3" t="n">
-        <v>-919.5561155150629</v>
-      </c>
-      <c r="P17" s="3" t="n">
-        <v>6237.286078798471</v>
-      </c>
-      <c r="Q17" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R17" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S17" s="3" t="n">
-        <v>-0</v>
+        <v>-861.6544573692352</v>
       </c>
       <c r="T17" s="3" t="n">
-        <v>-1559.321519699618</v>
+        <v>6297.930077842452</v>
       </c>
       <c r="U17" s="3" t="n">
-        <v>4677.964559098853</v>
+        <v>-0</v>
       </c>
       <c r="V17" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W17" s="4" t="n">
+      <c r="W17" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X17" s="3" t="n">
+        <v>-1574.482519460613</v>
+      </c>
+      <c r="Y17" s="3" t="n">
+        <v>4723.447558381839</v>
+      </c>
+      <c r="Z17" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA17" s="4" t="n">
         <v>0.3387345977965976</v>
       </c>
-      <c r="X17" s="3" t="n">
-        <v>1584.588443433088</v>
-      </c>
-      <c r="Y17" s="3" t="n">
-        <v>-4896.455533134445</v>
-      </c>
-      <c r="Z17" s="3" t="n">
-        <v>1498.392957231207</v>
+      <c r="AB17" s="3" t="n">
+        <v>1599.995108901793</v>
+      </c>
+      <c r="AC17" s="3" t="n">
+        <v>-4945.345699176984</v>
+      </c>
+      <c r="AD17" s="3" t="n">
+        <v>1512.129650594695</v>
       </c>
     </row>
     <row r="18">
@@ -2087,70 +2303,82 @@
         <v>158182.882238081</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>4382.891707768424</v>
+        <v>19578.2920264318</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>195781.1526663144</v>
+        <v>180585.7523476511</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1423.544327179952</v>
+        <v>1414.749947883118</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>8526.195100424382</v>
+        <v>8538.044840816387</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>-431.9023299103128</v>
+        <v>0</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>9949.739427604334</v>
+        <v>0</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>-369.5186905605743</v>
+        <v>0</v>
       </c>
       <c r="M18" s="3" t="n">
+        <v>-407.78214834861</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>9952.794788699504</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>-369.8167925903178</v>
+      </c>
+      <c r="P18" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N18" s="3" t="n">
+      <c r="Q18" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R18" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O18" s="3" t="n">
-        <v>-917.4683801319949</v>
-      </c>
-      <c r="P18" s="3" t="n">
-        <v>6211.252356911766</v>
-      </c>
-      <c r="Q18" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R18" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S18" s="3" t="n">
-        <v>-0</v>
+        <v>-859.725858921074</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>-1552.813089227941</v>
+        <v>6271.752137188112</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>4658.439267683824</v>
+        <v>-0</v>
       </c>
       <c r="V18" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W18" s="4" t="n">
+      <c r="W18" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X18" s="3" t="n">
+        <v>-1567.938034297028</v>
+      </c>
+      <c r="Y18" s="3" t="n">
+        <v>4703.814102891084</v>
+      </c>
+      <c r="Z18" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA18" s="4" t="n">
         <v>0.3165743904641098</v>
       </c>
-      <c r="X18" s="3" t="n">
-        <v>1474.742571681081</v>
-      </c>
-      <c r="Y18" s="3" t="n">
-        <v>-4997.354276667663</v>
-      </c>
-      <c r="Z18" s="3" t="n">
-        <v>1435.021933590194</v>
+      <c r="AB18" s="3" t="n">
+        <v>1489.107082479228</v>
+      </c>
+      <c r="AC18" s="3" t="n">
+        <v>-5047.347523462459</v>
+      </c>
+      <c r="AD18" s="3" t="n">
+        <v>1448.149885870148</v>
       </c>
     </row>
     <row r="19">
@@ -2169,70 +2397,82 @@
         <v>157708.3335913667</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>4247.6597086248</v>
+        <v>19401.16377208865</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>195231.9302080638</v>
+        <v>180078.4261446</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>1417.467968217985</v>
+        <v>1408.709549634254</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>8503.133256845873</v>
+        <v>8514.961630417523</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>-430.8432327721928</v>
+        <v>0</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>9920.601225063858</v>
+        <v>0</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>-368.4746896381946</v>
+        <v>0</v>
       </c>
       <c r="M19" s="3" t="n">
+        <v>-406.7631259987608</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>9923.671180051777</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>-368.7726562093861</v>
+      </c>
+      <c r="P19" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N19" s="3" t="n">
+      <c r="Q19" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R19" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O19" s="3" t="n">
-        <v>-915.3813347906425</v>
-      </c>
-      <c r="P19" s="3" t="n">
-        <v>6185.24520063502</v>
-      </c>
-      <c r="Q19" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R19" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S19" s="3" t="n">
-        <v>-0</v>
+        <v>-857.7980193494798</v>
       </c>
       <c r="T19" s="3" t="n">
-        <v>-1546.311300158755</v>
+        <v>6245.600504492911</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>4638.933900476266</v>
+        <v>-0</v>
       </c>
       <c r="V19" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W19" s="4" t="n">
+      <c r="W19" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X19" s="3" t="n">
+        <v>-1561.400126123228</v>
+      </c>
+      <c r="Y19" s="3" t="n">
+        <v>4684.200378369684</v>
+      </c>
+      <c r="Z19" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA19" s="4" t="n">
         <v>0.295863916321598</v>
       </c>
-      <c r="X19" s="3" t="n">
-        <v>1372.493151351934</v>
-      </c>
-      <c r="Y19" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z19" s="3" t="n">
-        <v>4638.933900476265</v>
+      <c r="AB19" s="3" t="n">
+        <v>1385.885868779566</v>
+      </c>
+      <c r="AC19" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD19" s="3" t="n">
+        <v>4684.200378369683</v>
       </c>
     </row>
     <row r="20">
@@ -2251,70 +2491,82 @@
         <v>157235.2085905927</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>4114.935374245784</v>
+        <v>19226.53346310066</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>194682.6732600421</v>
+        <v>179571.0751711872</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>1411.401811665745</v>
+        <v>1402.679232094721</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>8480.080866636248</v>
+        <v>8491.887698439497</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>-429.7831701646055</v>
+        <v>0</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>9891.482678301994</v>
+        <v>0</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>-367.4312708987649</v>
+        <v>0</v>
       </c>
       <c r="M20" s="3" t="n">
+        <v>-405.7433859173716</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>9894.566930534218</v>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>-367.7290925794743</v>
+      </c>
+      <c r="P20" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N20" s="3" t="n">
+      <c r="Q20" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R20" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O20" s="3" t="n">
-        <v>-913.29415838816</v>
-      </c>
-      <c r="P20" s="3" t="n">
-        <v>6159.257249015069</v>
-      </c>
-      <c r="Q20" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R20" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S20" s="3" t="n">
-        <v>-0</v>
+        <v>-855.8700856505114</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>-1539.814312253767</v>
+        <v>6219.467752304232</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>4619.442936761301</v>
+        <v>-0</v>
       </c>
       <c r="V20" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W20" s="4" t="n">
+      <c r="W20" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X20" s="3" t="n">
+        <v>-1554.866938076058</v>
+      </c>
+      <c r="Y20" s="3" t="n">
+        <v>4664.600814228173</v>
+      </c>
+      <c r="Z20" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA20" s="4" t="n">
         <v>0.2765083330108392</v>
       </c>
-      <c r="X20" s="3" t="n">
-        <v>1277.314465882563</v>
-      </c>
-      <c r="Y20" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z20" s="3" t="n">
-        <v>4619.4429367613</v>
+      <c r="AB20" s="3" t="n">
+        <v>1289.800995303236</v>
+      </c>
+      <c r="AC20" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD20" s="3" t="n">
+        <v>4664.600814228173</v>
       </c>
     </row>
     <row r="21">
@@ -2333,70 +2585,82 @@
         <v>156763.5029648209</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>3984.653642132095</v>
+        <v>19054.30860652376</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>194133.4373661655</v>
+        <v>179063.7824017739</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1405.347388756377</v>
+        <v>1396.660584274566</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>8457.044143672169</v>
+        <v>8468.829299986883</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>-428.7222799928859</v>
+        <v>0</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>9862.391532428546</v>
+        <v>0</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>-366.3887135220143</v>
+        <v>0</v>
       </c>
       <c r="M21" s="3" t="n">
+        <v>-404.7231012611575</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>9865.489884261448</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>-366.6863836849666</v>
+      </c>
+      <c r="P21" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N21" s="3" t="n">
+      <c r="Q21" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R21" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O21" s="3" t="n">
-        <v>-911.207061991429</v>
-      </c>
-      <c r="P21" s="3" t="n">
-        <v>6133.295756915102</v>
-      </c>
-      <c r="Q21" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R21" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S21" s="3" t="n">
-        <v>-0</v>
+        <v>-853.9423731267408</v>
       </c>
       <c r="T21" s="3" t="n">
-        <v>-1533.323939228776</v>
+        <v>6193.361127449741</v>
       </c>
       <c r="U21" s="3" t="n">
-        <v>4599.971817686327</v>
+        <v>-0</v>
       </c>
       <c r="V21" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W21" s="4" t="n">
+      <c r="W21" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X21" s="3" t="n">
+        <v>-1548.340281862435</v>
+      </c>
+      <c r="Y21" s="3" t="n">
+        <v>4645.020845587305</v>
+      </c>
+      <c r="Z21" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA21" s="4" t="n">
         <v>0.2584190028138684</v>
       </c>
-      <c r="X21" s="3" t="n">
-        <v>1188.720130098398</v>
-      </c>
-      <c r="Y21" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z21" s="3" t="n">
-        <v>4599.971817686326</v>
+      <c r="AB21" s="3" t="n">
+        <v>1200.361654966303</v>
+      </c>
+      <c r="AC21" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD21" s="3" t="n">
+        <v>4645.020845587304</v>
       </c>
     </row>
     <row r="22">
@@ -2415,70 +2679,82 @@
         <v>156293.2124559264</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>3856.965154353363</v>
+        <v>18884.60879521237</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>193584.0624048325</v>
+        <v>178556.4187639734</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>1399.302784858255</v>
+        <v>1390.651719809246</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>8434.016978172598</v>
+        <v>8445.780365886347</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>-427.660233179436</v>
+        <v>0</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>9833.319763030853</v>
+        <v>0</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>-365.3467348240691</v>
+        <v>0</v>
       </c>
       <c r="M22" s="3" t="n">
+        <v>-403.702009209128</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>9836.432085695593</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>-365.6442490316388</v>
+      </c>
+      <c r="P22" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N22" s="3" t="n">
+      <c r="Q22" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R22" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O22" s="3" t="n">
-        <v>-909.1194371383633</v>
-      </c>
-      <c r="P22" s="3" t="n">
-        <v>6107.35359106842</v>
-      </c>
-      <c r="Q22" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R22" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S22" s="3" t="n">
-        <v>-0</v>
+        <v>-852.014391303099</v>
       </c>
       <c r="T22" s="3" t="n">
-        <v>-1526.838397767105</v>
+        <v>6167.273445360855</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>4580.515193301316</v>
+        <v>-0</v>
       </c>
       <c r="V22" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W22" s="4" t="n">
+      <c r="W22" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X22" s="3" t="n">
+        <v>-1541.818361340214</v>
+      </c>
+      <c r="Y22" s="3" t="n">
+        <v>4625.455084020642</v>
+      </c>
+      <c r="Z22" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA22" s="4" t="n">
         <v>0.2415130867419331</v>
       </c>
-      <c r="X22" s="3" t="n">
-        <v>1106.254363202523</v>
-      </c>
-      <c r="Y22" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z22" s="3" t="n">
-        <v>4580.515193301315</v>
+      <c r="AB22" s="3" t="n">
+        <v>1117.107934927993</v>
+      </c>
+      <c r="AC22" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD22" s="3" t="n">
+        <v>4625.455084020641</v>
       </c>
     </row>
     <row r="23">
@@ -2497,70 +2773,82 @@
         <v>155824.3328185586</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>3731.775147623866</v>
+        <v>18717.37515743465</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>193034.6336986779</v>
+        <v>178049.0336888671</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1393.267620518527</v>
+        <v>1384.652223205568</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>8410.996220487734</v>
+        <v>8422.737740947969</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>-426.5971756689805</v>
+        <v>0</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>9804.263841006261</v>
+        <v>0</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>-364.3052012298799</v>
+        <v>0</v>
       </c>
       <c r="M23" s="3" t="n">
+        <v>-402.6801956052437</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>9807.389964153537</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>-364.6025541020302</v>
+      </c>
+      <c r="P23" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N23" s="3" t="n">
+      <c r="Q23" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R23" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O23" s="3" t="n">
-        <v>-907.0316080549759</v>
-      </c>
-      <c r="P23" s="3" t="n">
-        <v>6081.427031721405</v>
-      </c>
-      <c r="Q23" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R23" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S23" s="3" t="n">
-        <v>-0</v>
+        <v>-850.0863280176948</v>
       </c>
       <c r="T23" s="3" t="n">
-        <v>-1520.356757930351</v>
+        <v>6141.201082033813</v>
       </c>
       <c r="U23" s="3" t="n">
-        <v>4561.070273791053</v>
+        <v>-0</v>
       </c>
       <c r="V23" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W23" s="4" t="n">
+      <c r="W23" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X23" s="3" t="n">
+        <v>-1535.300270508453</v>
+      </c>
+      <c r="Y23" s="3" t="n">
+        <v>4605.90081152536</v>
+      </c>
+      <c r="Z23" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA23" s="4" t="n">
         <v>0.2257131651793767</v>
       </c>
-      <c r="X23" s="3" t="n">
-        <v>1029.493608102945</v>
-      </c>
-      <c r="Y23" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z23" s="3" t="n">
-        <v>4561.070273791052</v>
+      <c r="AB23" s="3" t="n">
+        <v>1039.612450671649</v>
+      </c>
+      <c r="AC23" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD23" s="3" t="n">
+        <v>4605.900811525359</v>
       </c>
     </row>
     <row r="24">
@@ -2579,70 +2867,82 @@
         <v>155356.859820103</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>3609.10780340419</v>
+        <v>18552.59467916774</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>192485.1176643032</v>
+        <v>177541.6307885396</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>1387.24251821494</v>
+        <v>1378.66271037507</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>8387.982908810223</v>
+        <v>8399.702371696925</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>-425.5330437526555</v>
+        <v>0</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>9775.225427025161</v>
+        <v>0</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>-363.2641667167077</v>
+        <v>0</v>
       </c>
       <c r="M24" s="3" t="n">
+        <v>-401.6576670289863</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>9778.365082071994</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>-363.5613490753784</v>
+      </c>
+      <c r="P24" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N24" s="3" t="n">
+      <c r="Q24" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R24" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O24" s="3" t="n">
-        <v>-904.943447124352</v>
-      </c>
-      <c r="P24" s="3" t="n">
-        <v>6055.517813184102</v>
-      </c>
-      <c r="Q24" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R24" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S24" s="3" t="n">
-        <v>-0</v>
+        <v>-848.1581969964504</v>
       </c>
       <c r="T24" s="3" t="n">
-        <v>-1513.879453296026</v>
+        <v>6115.145536000165</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>4541.638359888077</v>
+        <v>-0</v>
       </c>
       <c r="V24" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W24" s="4" t="n">
+      <c r="W24" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X24" s="3" t="n">
+        <v>-1528.786384000041</v>
+      </c>
+      <c r="Y24" s="3" t="n">
+        <v>4586.359152000124</v>
+      </c>
+      <c r="Z24" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA24" s="4" t="n">
         <v>0.2109468833452119</v>
       </c>
-      <c r="X24" s="3" t="n">
-        <v>958.0444572994495</v>
-      </c>
-      <c r="Y24" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z24" s="3" t="n">
-        <v>4541.638359888076</v>
+      <c r="AB24" s="3" t="n">
+        <v>967.4781690162149</v>
+      </c>
+      <c r="AC24" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD24" s="3" t="n">
+        <v>4586.359152000123</v>
       </c>
     </row>
     <row r="25">
@@ -2661,70 +2961,82 @@
         <v>154890.7892406426</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>3488.664404047545</v>
+        <v>18389.99300807812</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>191935.8036559615</v>
+        <v>177034.4750519309</v>
       </c>
       <c r="G25" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>1381.230315690886</v>
+        <v>1372.686040170388</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>8364.988944219192</v>
+        <v>8376.686240183277</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>-424.4684942941648</v>
+        <v>0</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>9746.219259910078</v>
+        <v>0</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>-362.2241640825854</v>
+        <v>0</v>
       </c>
       <c r="M25" s="3" t="n">
+        <v>-400.6350209971355</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>9749.372280353664</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>-362.5211704107389</v>
+      </c>
+      <c r="P25" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N25" s="3" t="n">
+      <c r="Q25" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R25" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O25" s="3" t="n">
-        <v>-902.8560538926536</v>
-      </c>
-      <c r="P25" s="3" t="n">
-        <v>6029.63904193484</v>
-      </c>
-      <c r="Q25" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R25" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S25" s="3" t="n">
-        <v>-0</v>
+        <v>-846.2310051973373</v>
       </c>
       <c r="T25" s="3" t="n">
-        <v>-1507.40976048371</v>
+        <v>6089.120104745587</v>
       </c>
       <c r="U25" s="3" t="n">
-        <v>4522.22928145113</v>
+        <v>-0</v>
       </c>
       <c r="V25" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W25" s="4" t="n">
+      <c r="W25" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X25" s="3" t="n">
+        <v>-1522.280026186397</v>
+      </c>
+      <c r="Y25" s="3" t="n">
+        <v>4566.84007855919</v>
+      </c>
+      <c r="Z25" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA25" s="4" t="n">
         <v>0.1971466199487961</v>
       </c>
-      <c r="X25" s="3" t="n">
-        <v>891.5422174715634</v>
-      </c>
-      <c r="Y25" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z25" s="3" t="n">
-        <v>4522.229281451129</v>
+      <c r="AB25" s="3" t="n">
+        <v>900.3370853346388</v>
+      </c>
+      <c r="AC25" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD25" s="3" t="n">
+        <v>4566.840078559189</v>
       </c>
     </row>
     <row r="26">
@@ -2743,70 +3055,82 @@
         <v>154426.1168729207</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>3370.531535764026</v>
+        <v>18229.61671857582</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>191386.5957624262</v>
+        <v>176527.5105796144</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>1375.230354459557</v>
+        <v>1366.721536749599</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>8342.013765364278</v>
+        <v>8353.688649602565</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>-423.4033269145679</v>
+        <v>0</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>9717.244119823834</v>
+        <v>0</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>-361.1851577037623</v>
+        <v>0</v>
       </c>
       <c r="M26" s="3" t="n">
+        <v>-399.6121478738718</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>9720.410186352163</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>-361.4819767190946</v>
+      </c>
+      <c r="P26" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N26" s="3" t="n">
+      <c r="Q26" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R26" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O26" s="3" t="n">
-        <v>-900.7690638972196</v>
-      </c>
-      <c r="P26" s="3" t="n">
-        <v>6003.789898222852</v>
-      </c>
-      <c r="Q26" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R26" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S26" s="3" t="n">
-        <v>-0</v>
+        <v>-844.3045402025349</v>
       </c>
       <c r="T26" s="3" t="n">
-        <v>-1500.947474555713</v>
+        <v>6063.123669430534</v>
       </c>
       <c r="U26" s="3" t="n">
-        <v>4502.842423667138</v>
+        <v>-0</v>
       </c>
       <c r="V26" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W26" s="4" t="n">
+      <c r="W26" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X26" s="3" t="n">
+        <v>-1515.780917357634</v>
+      </c>
+      <c r="Y26" s="3" t="n">
+        <v>4547.3427520729</v>
+      </c>
+      <c r="Z26" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA26" s="4" t="n">
         <v>0.1842491775222393</v>
       </c>
-      <c r="X26" s="3" t="n">
-        <v>829.6450130729171</v>
-      </c>
-      <c r="Y26" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z26" s="3" t="n">
-        <v>4502.842423667137</v>
+      <c r="AB26" s="3" t="n">
+        <v>837.8441619811483</v>
+      </c>
+      <c r="AC26" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD26" s="3" t="n">
+        <v>4547.342752072899</v>
       </c>
     </row>
     <row r="27">
@@ -2825,70 +3149,82 @@
         <v>153962.8385223019</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>3254.8177596427</v>
+        <v>18071.57195955784</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>190837.3761358024</v>
+        <v>176020.6219358873</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>1369.242085734736</v>
+        <v>1360.768677477932</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>8319.053211628054</v>
+        <v>8330.705544134587</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>-422.3372590840319</v>
+        <v>0</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>9688.295297362789</v>
+        <v>0</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>-360.1469701798169</v>
+        <v>0</v>
       </c>
       <c r="M27" s="3" t="n">
+        <v>-398.5887682154884</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>9691.474221612518</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>-360.4435953149421</v>
+      </c>
+      <c r="P27" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N27" s="3" t="n">
+      <c r="Q27" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R27" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O27" s="3" t="n">
-        <v>-898.6820293160492</v>
-      </c>
-      <c r="P27" s="3" t="n">
-        <v>5977.966297866924</v>
-      </c>
-      <c r="Q27" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R27" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S27" s="3" t="n">
-        <v>-0</v>
+        <v>-842.3783633563716</v>
       </c>
       <c r="T27" s="3" t="n">
-        <v>-1494.491574466731</v>
+        <v>6037.152262941205</v>
       </c>
       <c r="U27" s="3" t="n">
-        <v>4483.474723400192</v>
+        <v>-0</v>
       </c>
       <c r="V27" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W27" s="4" t="n">
+      <c r="W27" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X27" s="3" t="n">
+        <v>-1509.288065735301</v>
+      </c>
+      <c r="Y27" s="3" t="n">
+        <v>4527.864197205904</v>
+      </c>
+      <c r="Z27" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA27" s="4" t="n">
         <v>0.1721954930114386</v>
       </c>
-      <c r="X27" s="3" t="n">
-        <v>772.0341404002196</v>
-      </c>
-      <c r="Y27" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z27" s="3" t="n">
-        <v>4483.474723400192</v>
+      <c r="AB27" s="3" t="n">
+        <v>779.6778077267124</v>
+      </c>
+      <c r="AC27" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD27" s="3" t="n">
+        <v>4527.864197205903</v>
       </c>
     </row>
     <row r="28">
@@ -2907,70 +3243,82 @@
         <v>153500.950006735</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>3141.436701561634</v>
+        <v>17915.77087245581</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>190288.2219014508</v>
+        <v>175513.8877305567</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>1363.266984365541</v>
+        <v>1354.828936114454</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>8296.111242001467</v>
+        <v>8307.740872793869</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>-421.2704733337021</v>
+        <v>0</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>9659.378226367007</v>
+        <v>0</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>-359.1097893673695</v>
+        <v>0</v>
       </c>
       <c r="M28" s="3" t="n">
+        <v>-397.565056036615</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>9662.569808908323</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>-359.4062136340438</v>
+      </c>
+      <c r="P28" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N28" s="3" t="n">
+      <c r="Q28" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R28" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O28" s="3" t="n">
-        <v>-896.5952432255132</v>
-      </c>
-      <c r="P28" s="3" t="n">
-        <v>5952.173193774124</v>
-      </c>
-      <c r="Q28" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R28" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S28" s="3" t="n">
-        <v>-0</v>
+        <v>-840.4527733761154</v>
       </c>
       <c r="T28" s="3" t="n">
-        <v>-1488.043298443531</v>
+        <v>6011.210821898163</v>
       </c>
       <c r="U28" s="3" t="n">
-        <v>4464.129895330593</v>
+        <v>-0</v>
       </c>
       <c r="V28" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W28" s="4" t="n">
+      <c r="W28" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X28" s="3" t="n">
+        <v>-1502.802705474541</v>
+      </c>
+      <c r="Y28" s="3" t="n">
+        <v>4508.408116423623</v>
+      </c>
+      <c r="Z28" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA28" s="4" t="n">
         <v>0.1609303673004099</v>
       </c>
-      <c r="X28" s="3" t="n">
-        <v>718.4140637322929</v>
-      </c>
-      <c r="Y28" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z28" s="3" t="n">
-        <v>4464.129895330592</v>
+      <c r="AB28" s="3" t="n">
+        <v>725.5397741162029</v>
+      </c>
+      <c r="AC28" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD28" s="3" t="n">
+        <v>4508.40811642362</v>
       </c>
     </row>
     <row r="29">
@@ -2989,70 +3337,82 @@
         <v>153040.4471567149</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>3030.675337377085</v>
+        <v>17762.46397419752</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>189738.8368726338</v>
+        <v>175007.0482358134</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>1357.301506156684</v>
+        <v>1348.898796916738</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>8273.180170015059</v>
+        <v>8284.786942823757</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>-420.2024139334379</v>
+        <v>0</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>9630.481676171743</v>
+        <v>0</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>-358.073236923736</v>
+        <v>0</v>
       </c>
       <c r="M29" s="3" t="n">
+        <v>-396.5405185188199</v>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>9633.685739740495</v>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>-358.3694536512851</v>
+      </c>
+      <c r="P29" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N29" s="3" t="n">
+      <c r="Q29" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R29" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O29" s="3" t="n">
-        <v>-894.5075801160084</v>
-      </c>
-      <c r="P29" s="3" t="n">
-        <v>5926.400859131998</v>
-      </c>
-      <c r="Q29" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R29" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S29" s="3" t="n">
-        <v>-0</v>
+        <v>-838.5267832960909</v>
       </c>
       <c r="T29" s="3" t="n">
-        <v>-1481.600214783</v>
+        <v>5985.289502793118</v>
       </c>
       <c r="U29" s="3" t="n">
-        <v>4444.800644348999</v>
+        <v>-0</v>
       </c>
       <c r="V29" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W29" s="4" t="n">
+      <c r="W29" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X29" s="3" t="n">
+        <v>-1496.32237569828</v>
+      </c>
+      <c r="Y29" s="3" t="n">
+        <v>4488.967127094838</v>
+      </c>
+      <c r="Z29" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA29" s="4" t="n">
         <v>0.1504022124302896</v>
       </c>
-      <c r="X29" s="3" t="n">
-        <v>668.5078507216664</v>
-      </c>
-      <c r="Y29" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z29" s="3" t="n">
-        <v>4444.800644348997</v>
+      <c r="AB29" s="3" t="n">
+        <v>675.1505874419049</v>
+      </c>
+      <c r="AC29" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD29" s="3" t="n">
+        <v>4488.967127094837</v>
       </c>
     </row>
     <row r="30">
@@ -3071,70 +3431,82 @@
         <v>152581.3258152447</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>2922.072758175968</v>
+        <v>17611.26086869081</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>189189.6727850983</v>
+        <v>174500.4846745835</v>
       </c>
       <c r="G30" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>1351.349182486591</v>
+        <v>1342.98177665823</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>8250.272355094976</v>
+        <v>8261.85619931886</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>-419.1340202409753</v>
+        <v>0</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>9601.621537581568</v>
+        <v>0</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>-357.0378778535309</v>
+        <v>0</v>
       </c>
       <c r="M30" s="3" t="n">
+        <v>-395.5159676486035</v>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>9604.837975977089</v>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>-357.3338835059189</v>
+      </c>
+      <c r="P30" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N30" s="3" t="n">
+      <c r="Q30" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R30" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O30" s="3" t="n">
-        <v>-892.4207565833735</v>
-      </c>
-      <c r="P30" s="3" t="n">
-        <v>5900.662903144663</v>
-      </c>
-      <c r="Q30" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R30" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S30" s="3" t="n">
-        <v>-0</v>
+        <v>-836.6018417634173</v>
       </c>
       <c r="T30" s="3" t="n">
-        <v>-1475.165725786166</v>
+        <v>5959.402250707754</v>
       </c>
       <c r="U30" s="3" t="n">
-        <v>4425.497177358497</v>
+        <v>-0</v>
       </c>
       <c r="V30" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W30" s="4" t="n">
+      <c r="W30" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X30" s="3" t="n">
+        <v>-1489.850562676939</v>
+      </c>
+      <c r="Y30" s="3" t="n">
+        <v>4469.551688030816</v>
+      </c>
+      <c r="Z30" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA30" s="4" t="n">
         <v>0.1405628153554109</v>
       </c>
-      <c r="X30" s="3" t="n">
-        <v>622.0603425969344</v>
-      </c>
-      <c r="Y30" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z30" s="3" t="n">
-        <v>4425.497177358495</v>
+      <c r="AB30" s="3" t="n">
+        <v>628.2527686461406</v>
+      </c>
+      <c r="AC30" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD30" s="3" t="n">
+        <v>4469.551688030814</v>
       </c>
     </row>
     <row r="31">
@@ -3153,70 +3525,82 @@
         <v>152123.5818377989</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>2815.598226448382</v>
+        <v>17462.15098927427</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>188640.75124074</v>
+        <v>173994.1984779141</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>1345.409222338168</v>
+        <v>1337.077047589497</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>8227.387232441915</v>
+        <v>8238.948015123371</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>-418.065377957388</v>
+        <v>0</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>9572.796454780086</v>
+        <v>0</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>-356.00367374444</v>
+        <v>0</v>
       </c>
       <c r="M31" s="3" t="n">
+        <v>-394.4914345906229</v>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>9576.025062712868</v>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>-356.2994615567248</v>
+      </c>
+      <c r="P31" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N31" s="3" t="n">
+      <c r="Q31" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R31" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O31" s="3" t="n">
-        <v>-890.334854714812</v>
-      </c>
-      <c r="P31" s="3" t="n">
-        <v>5874.957926320833</v>
-      </c>
-      <c r="Q31" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R31" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S31" s="3" t="n">
-        <v>-0</v>
+        <v>-834.6779542160735</v>
       </c>
       <c r="T31" s="3" t="n">
-        <v>-1468.739481580208</v>
+        <v>5933.54764694007</v>
       </c>
       <c r="U31" s="3" t="n">
-        <v>4406.218444740625</v>
+        <v>-0</v>
       </c>
       <c r="V31" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W31" s="4" t="n">
+      <c r="W31" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X31" s="3" t="n">
+        <v>-1483.386911735018</v>
+      </c>
+      <c r="Y31" s="3" t="n">
+        <v>4450.160735205052</v>
+      </c>
+      <c r="Z31" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA31" s="4" t="n">
         <v>0.1313671171545896</v>
       </c>
-      <c r="X31" s="3" t="n">
-        <v>578.8322146389553</v>
-      </c>
-      <c r="Y31" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z31" s="3" t="n">
-        <v>4406.218444740623</v>
+      <c r="AB31" s="3" t="n">
+        <v>584.6047866584366</v>
+      </c>
+      <c r="AC31" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD31" s="3" t="n">
+        <v>4450.160735205051</v>
       </c>
     </row>
     <row r="32">
@@ -3235,70 +3619,82 @@
         <v>151667.2110922855</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>2711.031625117058</v>
+        <v>17314.90867524686</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>188092.283258411</v>
+        <v>173488.4062082812</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1339.485178407731</v>
+        <v>1331.188157500674</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>8204.537403274049</v>
+        <v>8216.074971882183</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>-416.9969580285589</v>
+        <v>0</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>9544.02258168178</v>
+        <v>0</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>-354.9711996991166</v>
+        <v>0</v>
       </c>
       <c r="M32" s="3" t="n">
+        <v>-393.4674040798284</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>9547.263129382858</v>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>-355.2667620253007</v>
+      </c>
+      <c r="P32" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N32" s="3" t="n">
+      <c r="Q32" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R32" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O32" s="3" t="n">
-        <v>-888.2506763819616</v>
-      </c>
-      <c r="P32" s="3" t="n">
-        <v>5849.300705600702</v>
-      </c>
-      <c r="Q32" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R32" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S32" s="3" t="n">
-        <v>-0</v>
+        <v>-832.7559435914684</v>
       </c>
       <c r="T32" s="3" t="n">
-        <v>-1462.325176400175</v>
+        <v>5907.740423766089</v>
       </c>
       <c r="U32" s="3" t="n">
-        <v>4386.975529200527</v>
+        <v>-0</v>
       </c>
       <c r="V32" s="3" t="n">
         <v>-0</v>
       </c>
-      <c r="W32" s="4" t="n">
+      <c r="W32" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="X32" s="3" t="n">
+        <v>-1476.935105941522</v>
+      </c>
+      <c r="Y32" s="3" t="n">
+        <v>4430.805317824566</v>
+      </c>
+      <c r="Z32" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA32" s="4" t="n">
         <v>0.1227730066865323</v>
       </c>
-      <c r="X32" s="3" t="n">
-        <v>538.6021759801901</v>
-      </c>
-      <c r="Y32" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z32" s="3" t="n">
-        <v>4386.975529200525</v>
+      <c r="AB32" s="3" t="n">
+        <v>543.9832909119986</v>
+      </c>
+      <c r="AC32" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD32" s="3" t="n">
+        <v>4430.805317824565</v>
       </c>
     </row>
     <row r="33">
@@ -3317,70 +3713,82 @@
         <v>151212.2094590087</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>2608.523789629269</v>
+        <v>17169.59528466741</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>187544.1089416657</v>
+        <v>172983.0374466276</v>
       </c>
       <c r="G33" s="3" t="n">
         <v>58</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>1333.576234217674</v>
+        <v>1325.314331153567</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>8181.721643435312</v>
+        <v>8193.235791873483</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>-415.9284150754938</v>
+        <v>0</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>9515.297877652985</v>
+        <v>0</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>-353.940390421766</v>
+        <v>0</v>
       </c>
       <c r="M33" s="3" t="n">
+        <v>-392.4437371240191</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>9518.550123027051</v>
+      </c>
+      <c r="O33" s="3" t="n">
+        <v>-354.2357182980107</v>
+      </c>
+      <c r="P33" s="3" t="n">
         <v>-2175</v>
       </c>
-      <c r="N33" s="3" t="n">
+      <c r="Q33" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="R33" s="3" t="n">
         <v>-276.5</v>
       </c>
-      <c r="O33" s="3" t="n">
-        <v>-886.1676139783295</v>
-      </c>
-      <c r="P33" s="3" t="n">
-        <v>5823.689873252889</v>
-      </c>
-      <c r="Q33" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="R33" s="3" t="n">
-        <v>-0</v>
-      </c>
       <c r="S33" s="3" t="n">
+        <v>-830.8355422971847</v>
+      </c>
+      <c r="T33" s="3" t="n">
+        <v>5881.978862431856</v>
+      </c>
+      <c r="U33" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="V33" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="W33" s="3" t="n">
         <v>-375</v>
       </c>
-      <c r="T33" s="3" t="n">
-        <v>-1362.172468313222</v>
-      </c>
-      <c r="U33" s="3" t="n">
-        <v>4086.517404939666</v>
-      </c>
-      <c r="V33" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="W33" s="4" t="n">
+      <c r="X33" s="3" t="n">
+        <v>-1376.744715607964</v>
+      </c>
+      <c r="Y33" s="3" t="n">
+        <v>4130.234146823892</v>
+      </c>
+      <c r="Z33" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AA33" s="4" t="n">
         <v>0.1147411277444227</v>
       </c>
-      <c r="X33" s="3" t="n">
-        <v>468.8916155899891</v>
-      </c>
-      <c r="Y33" s="3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Z33" s="3" t="n">
-        <v>4086.517404939665</v>
+      <c r="AB33" s="3" t="n">
+        <v>473.9077238550971</v>
+      </c>
+      <c r="AC33" s="3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD33" s="3" t="n">
+        <v>4130.23414682389</v>
       </c>
     </row>
     <row r="35">

</xml_diff>